<commit_message>
dash: fix KPI references, numeric month feed, Pos note
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Mazandasht_v03/08_Dash.xlsx
+++ b/Mazandasht_v03/08_Dash.xlsx
@@ -27,7 +27,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="0">Dash!$A$1:$H$63</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="6">'F1'!$A$1:$O$1809</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="7">'F2'!$A$1:$L$293</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="9">Help!$A$1:$H$33</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="9">Help!$A$1:$H$34</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="4">Ops!$A$1:$G$33</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="5">Parties!$A$1:$F$61</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">Pos!$A$1:$H$62</definedName>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="232">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="233">
   <si>
     <t xml:space="preserve">   مازندشت  ·  سورتینگ و بسته‌بندی مرکبات    ·    MAZANDASHT · CITRUS SORTING &amp; PACKING</t>
   </si>
@@ -725,13 +725,16 @@
     <t xml:space="preserve">کارت‌های بالای صفحه    </t>
   </si>
   <si>
-    <t xml:space="preserve">     •  وزن ورود / وزن خروج: جمع وزن خالص عملیات باسکول در کل دوره.</t>
+    <t xml:space="preserve">     •  کل وزن (kg): جمع وزن خالص همه ردیف‌های باسکول در کل دوره — همان عدد شیت Time.</t>
   </si>
   <si>
-    <t xml:space="preserve">     •  مبلغ خرید / مبلغ فروش: جمع مبلغ ردیف‌های خرید و فروش دفتر.</t>
+    <t xml:space="preserve">     •  کل مبلغ: جمع مبلغ تمام ردیف‌های دفتر (خرید، فروش، هزینه و …).</t>
   </si>
   <si>
-    <t xml:space="preserve">     •  اختلاف پز: پز ثبت‌شده منهای واریزی روز بعد؛ باید نزدیک صفر باشد.</t>
+    <t xml:space="preserve">     •  جمع بدهکار: جمع ستون بدهکار دفتر؛ در ثبت دوطرفه با جمع بستانکار برابر است.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     •  اختلاف پز: پز ثبت‌شده منهای واریزی ۲۰۰۶ و دریافتی باسکول دیگران؛ باید نزدیک صفر باشد.</t>
   </si>
   <si>
     <t xml:space="preserve">شیت Pos    </t>
@@ -9523,7 +9526,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8" ht="6" customHeight="1">
@@ -9682,43 +9685,43 @@
       <c r="G15" s="63"/>
       <c r="H15" s="63"/>
     </row>
-    <row r="17" spans="1:8" ht="26.25" customHeight="1">
-      <c r="A17" s="11" t="s">
+    <row r="16" spans="1:8" ht="26.25" customHeight="1">
+      <c r="A16" s="63" t="s">
         <v>219</v>
       </c>
-      <c r="B17" s="11"/>
-      <c r="C17" s="11"/>
-      <c r="D17" s="11"/>
-      <c r="E17" s="11"/>
-      <c r="F17" s="11"/>
-      <c r="G17" s="12" t="s">
+      <c r="B16" s="63"/>
+      <c r="C16" s="63"/>
+      <c r="D16" s="63"/>
+      <c r="E16" s="63"/>
+      <c r="F16" s="63"/>
+      <c r="G16" s="63"/>
+      <c r="H16" s="63"/>
+    </row>
+    <row r="18" spans="1:8" ht="26.25" customHeight="1">
+      <c r="A18" s="11" t="s">
+        <v>220</v>
+      </c>
+      <c r="B18" s="11"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="11"/>
+      <c r="F18" s="11"/>
+      <c r="G18" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="H17" s="12"/>
-    </row>
-    <row r="18" spans="1:8" ht="32.25" customHeight="1">
-      <c r="A18" s="62" t="s">
-        <v>220</v>
-      </c>
-      <c r="B18" s="62"/>
-      <c r="C18" s="62"/>
-      <c r="D18" s="62"/>
-      <c r="E18" s="62"/>
-      <c r="F18" s="62"/>
-      <c r="G18" s="62"/>
-      <c r="H18" s="62"/>
-    </row>
-    <row r="19" spans="1:8" ht="26.25" customHeight="1">
-      <c r="A19" s="63" t="s">
+      <c r="H18" s="12"/>
+    </row>
+    <row r="19" spans="1:8" ht="32.25" customHeight="1">
+      <c r="A19" s="62" t="s">
         <v>221</v>
       </c>
-      <c r="B19" s="63"/>
-      <c r="C19" s="63"/>
-      <c r="D19" s="63"/>
-      <c r="E19" s="63"/>
-      <c r="F19" s="63"/>
-      <c r="G19" s="63"/>
-      <c r="H19" s="63"/>
+      <c r="B19" s="62"/>
+      <c r="C19" s="62"/>
+      <c r="D19" s="62"/>
+      <c r="E19" s="62"/>
+      <c r="F19" s="62"/>
+      <c r="G19" s="62"/>
+      <c r="H19" s="62"/>
     </row>
     <row r="20" spans="1:8" ht="26.25" customHeight="1">
       <c r="A20" s="63" t="s">
@@ -9732,31 +9735,31 @@
       <c r="G20" s="63"/>
       <c r="H20" s="63"/>
     </row>
-    <row r="22" spans="1:8" ht="26.25" customHeight="1">
-      <c r="A22" s="11" t="s">
+    <row r="21" spans="1:8" ht="26.25" customHeight="1">
+      <c r="A21" s="63" t="s">
         <v>223</v>
       </c>
-      <c r="B22" s="11"/>
-      <c r="C22" s="11"/>
-      <c r="D22" s="11"/>
-      <c r="E22" s="11"/>
-      <c r="F22" s="11"/>
-      <c r="G22" s="12" t="s">
+      <c r="B21" s="63"/>
+      <c r="C21" s="63"/>
+      <c r="D21" s="63"/>
+      <c r="E21" s="63"/>
+      <c r="F21" s="63"/>
+      <c r="G21" s="63"/>
+      <c r="H21" s="63"/>
+    </row>
+    <row r="23" spans="1:8" ht="26.25" customHeight="1">
+      <c r="A23" s="11" t="s">
+        <v>224</v>
+      </c>
+      <c r="B23" s="11"/>
+      <c r="C23" s="11"/>
+      <c r="D23" s="11"/>
+      <c r="E23" s="11"/>
+      <c r="F23" s="11"/>
+      <c r="G23" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="H22" s="12"/>
-    </row>
-    <row r="23" spans="1:8" ht="26.25" customHeight="1">
-      <c r="A23" s="63" t="s">
-        <v>224</v>
-      </c>
-      <c r="B23" s="63"/>
-      <c r="C23" s="63"/>
-      <c r="D23" s="63"/>
-      <c r="E23" s="63"/>
-      <c r="F23" s="63"/>
-      <c r="G23" s="63"/>
-      <c r="H23" s="63"/>
+      <c r="H23" s="12"/>
     </row>
     <row r="24" spans="1:8" ht="26.25" customHeight="1">
       <c r="A24" s="63" t="s">
@@ -9770,31 +9773,31 @@
       <c r="G24" s="63"/>
       <c r="H24" s="63"/>
     </row>
-    <row r="26" spans="1:8" ht="26.25" customHeight="1">
-      <c r="A26" s="11" t="s">
+    <row r="25" spans="1:8" ht="26.25" customHeight="1">
+      <c r="A25" s="63" t="s">
         <v>226</v>
       </c>
-      <c r="B26" s="11"/>
-      <c r="C26" s="11"/>
-      <c r="D26" s="11"/>
-      <c r="E26" s="11"/>
-      <c r="F26" s="11"/>
-      <c r="G26" s="12" t="s">
+      <c r="B25" s="63"/>
+      <c r="C25" s="63"/>
+      <c r="D25" s="63"/>
+      <c r="E25" s="63"/>
+      <c r="F25" s="63"/>
+      <c r="G25" s="63"/>
+      <c r="H25" s="63"/>
+    </row>
+    <row r="27" spans="1:8" ht="26.25" customHeight="1">
+      <c r="A27" s="11" t="s">
+        <v>227</v>
+      </c>
+      <c r="B27" s="11"/>
+      <c r="C27" s="11"/>
+      <c r="D27" s="11"/>
+      <c r="E27" s="11"/>
+      <c r="F27" s="11"/>
+      <c r="G27" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="H26" s="12"/>
-    </row>
-    <row r="27" spans="1:8" ht="26.25" customHeight="1">
-      <c r="A27" s="63" t="s">
-        <v>227</v>
-      </c>
-      <c r="B27" s="63"/>
-      <c r="C27" s="63"/>
-      <c r="D27" s="63"/>
-      <c r="E27" s="63"/>
-      <c r="F27" s="63"/>
-      <c r="G27" s="63"/>
-      <c r="H27" s="63"/>
+      <c r="H27" s="12"/>
     </row>
     <row r="28" spans="1:8" ht="26.25" customHeight="1">
       <c r="A28" s="63" t="s">
@@ -9808,34 +9811,46 @@
       <c r="G28" s="63"/>
       <c r="H28" s="63"/>
     </row>
-    <row r="30" spans="1:8" ht="26.25" customHeight="1">
-      <c r="A30" s="11" t="s">
+    <row r="29" spans="1:8" ht="26.25" customHeight="1">
+      <c r="A29" s="63" t="s">
         <v>229</v>
       </c>
-      <c r="B30" s="11"/>
-      <c r="C30" s="11"/>
-      <c r="D30" s="11"/>
-      <c r="E30" s="11"/>
-      <c r="F30" s="11"/>
-      <c r="G30" s="12" t="s">
+      <c r="B29" s="63"/>
+      <c r="C29" s="63"/>
+      <c r="D29" s="63"/>
+      <c r="E29" s="63"/>
+      <c r="F29" s="63"/>
+      <c r="G29" s="63"/>
+      <c r="H29" s="63"/>
+    </row>
+    <row r="31" spans="1:8" ht="26.25" customHeight="1">
+      <c r="A31" s="11" t="s">
         <v>230</v>
       </c>
-      <c r="H30" s="12"/>
-    </row>
-    <row r="31" spans="1:8" ht="32.25" customHeight="1">
-      <c r="A31" s="62" t="s">
+      <c r="B31" s="11"/>
+      <c r="C31" s="11"/>
+      <c r="D31" s="11"/>
+      <c r="E31" s="11"/>
+      <c r="F31" s="11"/>
+      <c r="G31" s="12" t="s">
         <v>231</v>
       </c>
-      <c r="B31" s="62"/>
-      <c r="C31" s="62"/>
-      <c r="D31" s="62"/>
-      <c r="E31" s="62"/>
-      <c r="F31" s="62"/>
-      <c r="G31" s="62"/>
-      <c r="H31" s="62"/>
+      <c r="H31" s="12"/>
+    </row>
+    <row r="32" spans="1:8" ht="32.25" customHeight="1">
+      <c r="A32" s="62" t="s">
+        <v>232</v>
+      </c>
+      <c r="B32" s="62"/>
+      <c r="C32" s="62"/>
+      <c r="D32" s="62"/>
+      <c r="E32" s="62"/>
+      <c r="F32" s="62"/>
+      <c r="G32" s="62"/>
+      <c r="H32" s="62"/>
     </row>
   </sheetData>
-  <mergeCells count="29">
+  <mergeCells count="30">
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A3:H3"/>
     <mergeCell ref="A4:H4"/>
@@ -9849,22 +9864,23 @@
     <mergeCell ref="A13:H13"/>
     <mergeCell ref="A14:H14"/>
     <mergeCell ref="A15:H15"/>
-    <mergeCell ref="A17:F17"/>
-    <mergeCell ref="G17:H17"/>
-    <mergeCell ref="A18:H18"/>
+    <mergeCell ref="A16:H16"/>
+    <mergeCell ref="A18:F18"/>
+    <mergeCell ref="G18:H18"/>
     <mergeCell ref="A19:H19"/>
     <mergeCell ref="A20:H20"/>
-    <mergeCell ref="A22:F22"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="A23:H23"/>
+    <mergeCell ref="A21:H21"/>
+    <mergeCell ref="A23:F23"/>
+    <mergeCell ref="G23:H23"/>
     <mergeCell ref="A24:H24"/>
-    <mergeCell ref="A26:F26"/>
-    <mergeCell ref="G26:H26"/>
-    <mergeCell ref="A27:H27"/>
+    <mergeCell ref="A25:H25"/>
+    <mergeCell ref="A27:F27"/>
+    <mergeCell ref="G27:H27"/>
     <mergeCell ref="A28:H28"/>
-    <mergeCell ref="A30:F30"/>
-    <mergeCell ref="G30:H30"/>
-    <mergeCell ref="A31:H31"/>
+    <mergeCell ref="A29:H29"/>
+    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="G31:H31"/>
+    <mergeCell ref="A32:H32"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.28" right="0.28" top="0.42" bottom="0.48" header="0.22" footer="0.22"/>

</xml_diff>